<commit_message>
Deployed 8e962d2 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/downloads/acces-format-publication.xlsx
+++ b/downloads/acces-format-publication.xlsx
@@ -453,27 +453,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Numérique</t>
+          <t>Papier</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Papier</t>
+          <t>Numérique</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Deployed d8f7dba with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/downloads/acces-format-publication.xlsx
+++ b/downloads/acces-format-publication.xlsx
@@ -460,7 +460,7 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -470,7 +470,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C3" t="n">
         <v>2</v>
@@ -483,10 +483,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C4" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>